<commit_message>
feat: implement System4 analysis engine and add comprehensive unit tests for bug investigation workflows
</commit_message>
<xml_diff>
--- a/fixtures/excel/column_mapping.xlsx
+++ b/fixtures/excel/column_mapping.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1365,22 +1365,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>tpaymentquality_old</t>
+          <t>tdupshipment_old</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>tpaymentquality_new</t>
+          <t>tdupshipment_new</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>payment_id</t>
+          <t>shipment_id</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>PaymentIdentifier</t>
+          <t>ShipmentIdentifier</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1407,32 +1407,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>tpaymentquality_old</t>
+          <t>tdupshipment_old</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>tpaymentquality_new</t>
+          <t>tdupshipment_new</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>payment_score</t>
+          <t>shipment_status</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>PaymentQualityIndex</t>
+          <t>ShipmentStatus</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
     </row>
@@ -1449,22 +1449,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tshipment_old</t>
+          <t>teventlog_old</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>tshipment_new</t>
+          <t>teventlog_new</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>shipment_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>ShipmentIdentifier</t>
+          <t>EventIdentifier</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1491,32 +1491,32 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>tshipment_old</t>
+          <t>teventlog_old</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>tshipment_new</t>
+          <t>teventlog_new</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>shpmnt_status</t>
+          <t>occurred_ts</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ShipmentStatus</t>
+          <t>EventOccurredTs</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp</t>
         </is>
       </c>
     </row>
@@ -1533,22 +1533,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>tbillingvariance_old</t>
+          <t>torderlink_old</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>tbillingvariance_new</t>
+          <t>torderlink_new</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>bill_id</t>
+          <t>order_id</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>BillingIdentifier</t>
+          <t>OrderIdentifier</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1575,32 +1575,32 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>tbillingvariance_old</t>
+          <t>torderlink_old</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>tbillingvariance_new</t>
+          <t>torderlink_new</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>invoice_variance</t>
+          <t>market_code</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>BillingVarianceAmount</t>
+          <t>RegionalMarketCode</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
     </row>
@@ -1617,22 +1617,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>tprofileaudit_old</t>
+          <t>torderlink_old</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>tprofileaudit_new</t>
+          <t>torderlink_new</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>profile_key</t>
+          <t>settlement_flag</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ProfileIdentifier</t>
+          <t>SettlementStatusCode</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1659,30 +1659,324 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>tpaymentquality_old</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>tpaymentquality_new</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>payment_id</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>PaymentIdentifier</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Gavin2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Gavin3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>tpaymentquality_old</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>tpaymentquality_new</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>payment_score</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>PaymentQualityIndex</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Gavin2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Gavin3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>tshipment_old</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>tshipment_new</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>shipment_id</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ShipmentIdentifier</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Gavin2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Gavin3</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>tshipment_old</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>tshipment_new</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>shpmnt_status</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ShipmentStatus</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Gavin2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Gavin3</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>tbillingvariance_old</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>tbillingvariance_new</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>bill_id</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>BillingIdentifier</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Gavin2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Gavin3</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>tbillingvariance_old</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>tbillingvariance_new</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>invoice_variance</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>BillingVarianceAmount</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Gavin2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Gavin3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>tprofileaudit_old</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>tprofileaudit_new</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>profile_key</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>ProfileIdentifier</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Gavin2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Gavin3</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>tprofileaudit_old</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>tprofileaudit_new</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>reviewed_on</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>ProfileGovernanceReviewTs</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>

</xml_diff>